<commit_message>
update file excel v2
</commit_message>
<xml_diff>
--- a/public/rooms.xlsx
+++ b/public/rooms.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbookprom1/Desktop/DEMO/web-home/public/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DB14E77-0020-EA4A-BF93-5EE9688B08D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47639335-9028-664D-8989-6357D42DAF80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="620" windowWidth="28800" windowHeight="16080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="40">
   <si>
     <t>id</t>
   </si>
@@ -94,39 +94,15 @@
     <t>Mới đăng</t>
   </si>
   <si>
-    <t>3.800đ / kWh</t>
-  </si>
-  <si>
-    <t>100.000đ / người</t>
-  </si>
-  <si>
     <t>Phòng mới, sạch sẽ, gần trường học và nhiều tiện ích.</t>
   </si>
   <si>
     <t>Máy lạnh | Thang máy | Camera an ninh</t>
   </si>
   <si>
-    <t>Căn hộ mini có ban công riêng</t>
-  </si>
-  <si>
-    <t>Bình Thạnh, TP. HCM</t>
-  </si>
-  <si>
-    <t>Đường Nguyễn Gia Trí, Bình Thạnh</t>
-  </si>
-  <si>
-    <t>https://images.unsplash.com/photo-1505693416388-ac5ce068fe85?auto=format&amp;fit=crop&amp;w=900&amp;q=80</t>
-  </si>
-  <si>
     <t>Còn phòng</t>
   </si>
   <si>
-    <t>150.000đ / người</t>
-  </si>
-  <si>
-    <t>120.000đ / xe</t>
-  </si>
-  <si>
     <t>Không gian riêng tư, nhiều ánh sáng và có ban công thoáng mát.</t>
   </si>
   <si>
@@ -136,21 +112,9 @@
     <t>Phòng trọ yên tĩnh, giờ giấc tự do</t>
   </si>
   <si>
-    <t>Hải Châu, Đà Nẵng</t>
-  </si>
-  <si>
-    <t>Đường Lê Thanh Nghị, Hải Châu, Đà Nẵng</t>
-  </si>
-  <si>
     <t>Giá tốt</t>
   </si>
   <si>
-    <t>3.500đ / kWh</t>
-  </si>
-  <si>
-    <t>80.000đ / xe</t>
-  </si>
-  <si>
     <t>Phòng yên tĩnh, phù hợp sinh viên và người đi làm.</t>
   </si>
   <si>
@@ -158,16 +122,42 @@
   </si>
   <si>
     <t>80/12/15A Dương Quảng Hàm - P5 - Gò Vấp</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/qang3dcs/image/upload/v1786600856/1WUpukiDjiqG0WyBAzxJXtzdLmnMXw9vtWbkitBERGX5dzK87YnuTaBsHfKfKVSgDSg.jpg</t>
+  </si>
+  <si>
+    <t>15/19 Đường C1 - P13 - Tân Bình</t>
+  </si>
+  <si>
+    <t>Tân bình, TP. HCM</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/qang3dcs/image/upload/v1786600988/1WUpukiE7Bht0S6s7ADvJyFsatJLUCql7rzOVAgrRNn8bZSmOPu5jgX4ne8DZhMnuBV.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1086 Cách Mạng Tháng Tám -P4 - Tân Bình </t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/qang3dcs/image/upload/v1786601199/1WUpukiEsHrqbxN6lOkqTnAGvw4SmMpklIN1j5JOnAA2bZHlbt2tOBbm3ubskcqfdaj.jpg</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -190,13 +180,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -644,7 +637,7 @@
         <v>14</v>
       </c>
       <c r="D3" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="E3">
         <v>5.2</v>
@@ -652,26 +645,26 @@
       <c r="F3">
         <v>24</v>
       </c>
-      <c r="G3" t="s">
-        <v>31</v>
+      <c r="G3" s="1" t="s">
+        <v>34</v>
       </c>
       <c r="H3" t="s">
         <v>23</v>
       </c>
       <c r="I3" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="J3" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="K3" t="s">
         <v>20</v>
       </c>
       <c r="L3" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="M3" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
@@ -679,40 +672,40 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="C4" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="D4" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="E4">
-        <v>4.9000000000000004</v>
+        <v>5.2</v>
       </c>
       <c r="F4">
         <v>28</v>
       </c>
-      <c r="G4" t="s">
-        <v>31</v>
+      <c r="G4" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="H4" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="I4" t="s">
         <v>18</v>
       </c>
       <c r="J4" t="s">
-        <v>33</v>
+        <v>19</v>
       </c>
       <c r="K4" t="s">
-        <v>34</v>
+        <v>20</v>
       </c>
       <c r="L4" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="M4" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
@@ -720,47 +713,52 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="C5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D5" t="s">
         <v>38</v>
       </c>
-      <c r="D5" t="s">
-        <v>39</v>
-      </c>
       <c r="E5">
-        <v>2.9</v>
+        <v>5.5</v>
       </c>
       <c r="F5">
         <v>20</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="H5" t="s">
+        <v>30</v>
+      </c>
+      <c r="I5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J5" t="s">
+        <v>19</v>
+      </c>
+      <c r="K5" t="s">
+        <v>20</v>
+      </c>
+      <c r="L5" t="s">
         <v>31</v>
       </c>
-      <c r="H5" t="s">
-        <v>40</v>
-      </c>
-      <c r="I5" t="s">
-        <v>41</v>
-      </c>
-      <c r="J5" t="s">
-        <v>25</v>
-      </c>
-      <c r="K5" t="s">
-        <v>42</v>
-      </c>
-      <c r="L5" t="s">
-        <v>43</v>
-      </c>
       <c r="M5" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="G3" r:id="rId1" xr:uid="{4FAFA07E-9AEA-5C45-A4EC-3AF14C8844CA}"/>
+    <hyperlink ref="G4" r:id="rId2" xr:uid="{27D91BE3-3306-D147-8EC2-6CBFC55515AC}"/>
+    <hyperlink ref="G5" r:id="rId3" xr:uid="{64C16A79-46C6-7348-9386-096247CB262A}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:M1 A4:M5 A2:D2 F2:M2 A3 F3 H3:M3" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:M1 A5:B5 A2:D2 F2:M2 A3 F3 H3 A4 F4 H4:I4 F5 H5 L4:M4 L5:M5 K3:M3" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>